<commit_message>
upload all scripts and plots including flight data and embedded code
</commit_message>
<xml_diff>
--- a/data/probability.xlsx
+++ b/data/probability.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://livemanchesterac-my.sharepoint.com/personal/rufus_clark_student_manchester_ac_uk/Documents/Documents/University/Year 3/Individual Project/code/models/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="146" documentId="8_{00659E19-EDB9-4A85-807C-1379F88B69EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CD73FE2D-D016-477B-880B-146617FD420B}"/>
+  <xr:revisionPtr revIDLastSave="152" documentId="8_{00659E19-EDB9-4A85-807C-1379F88B69EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A3A0FD61-9C85-41A9-B0CC-58B219E6E563}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="12980" windowHeight="16090" activeTab="1" xr2:uid="{3AC71859-7A47-46AF-AB5E-931F34361CA9}"/>
+    <workbookView xWindow="12710" yWindow="0" windowWidth="12980" windowHeight="16090" activeTab="1" xr2:uid="{3AC71859-7A47-46AF-AB5E-931F34361CA9}"/>
   </bookViews>
   <sheets>
     <sheet name="working" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="32">
   <si>
     <t>Failure Rate - Simple</t>
   </si>
@@ -130,6 +130,9 @@
   </si>
   <si>
     <t>N/A</t>
+  </si>
+  <si>
+    <t>no recovery device deployed</t>
   </si>
 </sst>
 </file>
@@ -138,7 +141,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0%"/>
-    <numFmt numFmtId="166" formatCode="0.000"/>
+    <numFmt numFmtId="165" formatCode="0.000"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -180,7 +183,7 @@
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1515,7 +1518,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{917029C2-11B2-45EB-A536-E7E9241AFDF4}">
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="43.26953125" bestFit="1" customWidth="1"/>
@@ -1825,12 +1828,64 @@
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
+        <v>31</v>
+      </c>
+      <c r="B7" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="2">
+        <f>working!B26</f>
+        <v>3.2000000000000001E-2</v>
+      </c>
+      <c r="D7" s="2">
+        <f>working!C26</f>
+        <v>0</v>
+      </c>
+      <c r="E7" s="2">
+        <f>working!D26</f>
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="F7" s="2">
+        <f>working!E26</f>
+        <v>1.7000000000000001E-2</v>
+      </c>
+      <c r="G7" s="2">
+        <f>working!F26</f>
+        <v>1.0999999999999999E-2</v>
+      </c>
+      <c r="H7" s="2">
+        <f>working!G26</f>
+        <v>1.0999999999999999E-2</v>
+      </c>
+      <c r="I7" s="2">
+        <f>working!H26</f>
+        <v>1.9E-2</v>
+      </c>
+      <c r="J7" s="2">
+        <f>working!I26</f>
+        <v>8.9999999999999993E-3</v>
+      </c>
+      <c r="K7" s="2">
+        <f>working!J26</f>
+        <v>7.0000000000000001E-3</v>
+      </c>
+      <c r="L7" s="2">
+        <f>working!K26</f>
+        <v>1.7000000000000001E-2</v>
+      </c>
+      <c r="M7" s="2">
+        <f>working!L26</f>
+        <v>1.7999999999999999E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
         <v>26</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B8" t="s">
         <v>17</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C8" t="s">
         <v>30</v>
       </c>
     </row>

</xml_diff>